<commit_message>
Add ability to import system roles and their permissions via Excel
Integrates a new "ROLES" sheet into the master Excel template, allowing for the import of system roles, their descriptions, colors, and associated module permissions. The backend logic in `importacion-maestro.ts` is updated to process this new sheet, create roles in `system_roles`, and assign permissions via `rol_permisos`, while validating module keys and handling duplicates.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 3f9a2cf7-4d64-4a60-a668-778e2b0553c6
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: cff8a8d8-e34b-49e6-8b14-2154b0b3e2bc
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/987b05e8-e17a-40f4-b366-3baeddd84475/3f9a2cf7-4d64-4a60-a668-778e2b0553c6/WXc2aeU
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/ISP_PlantillaMaestra_CargaInicial.xlsx
+++ b/ISP_PlantillaMaestra_CargaInicial.xlsx
@@ -15,7 +15,8 @@
     <sheet name="ANTICIPOS" sheetId="10" r:id="rId10"/>
     <sheet name="HISTORIAL_PRESTACIONES" sheetId="11" r:id="rId11"/>
     <sheet name="USUARIOS" sheetId="12" r:id="rId12"/>
-    <sheet name="IGSS_PATRONO" sheetId="13" r:id="rId13"/>
+    <sheet name="ROLES" sheetId="13" r:id="rId13"/>
+    <sheet name="IGSS_PATRONO" sheetId="14" r:id="rId14"/>
   </sheets>
 </workbook>
 </file>
@@ -409,7 +410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A32"/>
+  <dimension ref="A1:A43"/>
   <cols>
     <col min="1" max="1" width="80.83203125" customWidth="1"/>
   </cols>
@@ -431,7 +432,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>• No cambie los nombres de las hojas (ej: COLABORADORES, CLIENTES)</v>
+        <v>• No cambie los nombres de las hojas</v>
       </c>
     </row>
     <row r="5">
@@ -461,7 +462,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>• Puede dejar filas vacías entre registros — se omitirán automáticamente</v>
+        <v>• Puede dejar filas vacías — se omitirán automáticamente</v>
       </c>
     </row>
     <row r="11">
@@ -471,7 +472,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ORDEN DE DEPENDENCIAS (no cambiar el orden de llenado)</v>
+        <v>ORDEN DE DEPENDENCIAS (llenar en este orden)</v>
       </c>
     </row>
     <row r="13">
@@ -491,7 +492,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v xml:space="preserve">  4. COLABORADORES — dependen de CLIENTES</v>
+        <v xml:space="preserve">  4. COLABORADORES — dependen de CLIENTES y PUESTOS</v>
       </c>
     </row>
     <row r="17">
@@ -531,52 +532,107 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v xml:space="preserve"> 12. IGSS_PATRONO — configuración única del patrono</v>
+        <v xml:space="preserve"> 12. ROLES — independiente (crea roles y asigna permisos)</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v/>
+        <v xml:space="preserve"> 13. IGSS_PATRONO — configuración única del patrono</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>REFERENCIAS CRUZADAS</v>
+        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v xml:space="preserve">  • En PUESTOS → cliente_nombre debe ser exactamente igual al nombre en CLIENTES</v>
+        <v>REFERENCIAS CRUZADAS</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v xml:space="preserve">  • En COLABORADORES → cliente_nombre debe ser exactamente igual al nombre en CLIENTES</v>
+        <v xml:space="preserve">  • En PUESTOS → cliente_nombre debe ser exactamente igual al nombre en CLIENTES</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v xml:space="preserve">  • En COLABORADORES → puesto_operativo debe ser exactamente igual al nombre en PUESTOS</v>
+        <v xml:space="preserve">  • En COLABORADORES → cliente_nombre debe ser exactamente igual al nombre en CLIENTES</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v xml:space="preserve">  • En ARMERIA/VEHICULOS → custodio_dpi es más confiable que custodio_nombre</v>
+        <v xml:space="preserve">  • En COLABORADORES → puesto_operativo debe ser exactamente igual al nombre en PUESTOS</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v xml:space="preserve">  • En ANTICIPOS/HISTORIAL → colaborador_dpi es más confiable que colaborador_nombre</v>
+        <v xml:space="preserve">  • En ARMERIA/VEHICULOS → custodio_dpi es más confiable que custodio_nombre</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
+        <v xml:space="preserve">  • En ANTICIPOS/HISTORIAL → colaborador_dpi es más confiable que colaborador_nombre</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
         <v xml:space="preserve">  • En USUARIOS → colaborador_dpi vincula el usuario al colaborador</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>MÓDULOS DISPONIBLES PARA ROLES (columna 'modulos' — separar por comas)</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v xml:space="preserve">  dashboard, pizarron, seguimiento_ssa, pipeline_ssa, tareas, incidencias</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v xml:space="preserve">  custodias, cambios_estructurales, clientes, comercial, reportes, kpi</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v xml:space="preserve">  empleados, reclutamiento, anticipos, eventos_rrhh, alertas_rrhh, nomina</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v xml:space="preserve">  pre_planilla, planilla, turnos, cambios_salariales, prestaciones</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v xml:space="preserve">  solicitudes_vacaciones, planillas_especiales, libro_salarios, igss_planilla</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v xml:space="preserve">  carnets_qr, kiosco_solicitudes, solicitudes_eliminacion, usuarios</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v xml:space="preserve">  config_whatsapp, cms, simulador_wa, bodega, vehiculos, armeria</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v xml:space="preserve">  importacion, control_qr</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A43"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1019,6 +1075,109 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E5"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="5" max="5" width="20.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>clave *</v>
+      </c>
+      <c r="B1" t="str">
+        <v>label *</v>
+      </c>
+      <c r="C1" t="str">
+        <v>descripcion</v>
+      </c>
+      <c r="D1" t="str">
+        <v>color</v>
+      </c>
+      <c r="E1" t="str">
+        <v>modulos</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>jefe_zona</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Jefe de Zona</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Supervisa operaciones de múltiples puestos en una zona</v>
+      </c>
+      <c r="D2" t="str">
+        <v>#10B981</v>
+      </c>
+      <c r="E2" t="str">
+        <v>dashboard,pizarron,empleados,clientes,eventos_rrhh,nomina,custodias</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v/>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v/>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v/>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E5"/>
   <cols>

</xml_diff>